<commit_message>
Add egg to lifestage
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v21.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v21.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{544E36C7-1BB8-954B-A3B3-D2226AFCBED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5048163F-507C-B844-9687-6556C59B4304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19460" activeTab="3" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="1" r:id="rId1"/>
@@ -911,9 +911,6 @@
     <t>Sex of the organism (e.g., male or female)</t>
   </si>
   <si>
-    <t xml:space="preserve">fry, larva, nymph, pupa, juvenile, or adult </t>
-  </si>
-  <si>
     <t>Journal Article, Book, Book Section, Report, Unpublished</t>
   </si>
   <si>
@@ -1062,6 +1059,9 @@
   </si>
   <si>
     <t>If there is no genus and species for the organism then use the next type of classifcation e.g., family ect. (Salvelinus); If validation does not return a valid scientific name and you have searched the taxonomic table but haven't found the species; please contact the database manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">egg, fry, larva, nymph, pupa, juvenile, or adult </t>
   </si>
 </sst>
 </file>
@@ -1386,13 +1386,13 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1747,20 +1747,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="47" t="s">
         <v>197</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="47" t="s">
         <v>166</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="22" t="s">
@@ -1860,7 +1860,7 @@
         <v>78</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F9" s="31"/>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="E12" s="31"/>
       <c r="F12" s="34" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="28" x14ac:dyDescent="0.2">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="E13" s="31"/>
       <c r="F13" s="34" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -2180,14 +2180,14 @@
         <v>6</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D29" s="31" t="s">
         <v>11</v>
       </c>
       <c r="E29" s="31"/>
       <c r="F29" s="34" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="112" x14ac:dyDescent="0.2">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="34" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -2256,7 +2256,7 @@
         <v>182</v>
       </c>
       <c r="E33" s="34" t="s">
-        <v>207</v>
+        <v>257</v>
       </c>
       <c r="F33" s="31"/>
     </row>
@@ -2274,7 +2274,7 @@
         <v>113</v>
       </c>
       <c r="E34" s="31" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F34" s="31"/>
     </row>
@@ -2286,10 +2286,10 @@
         <v>160</v>
       </c>
       <c r="C35" s="31" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D35" s="34" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E35" s="31"/>
       <c r="F35" s="31"/>
@@ -2302,7 +2302,7 @@
         <v>173</v>
       </c>
       <c r="C36" s="31" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D36" s="31" t="s">
         <v>40</v>
@@ -2318,7 +2318,7 @@
         <v>99</v>
       </c>
       <c r="C37" s="31" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D37" s="31" t="s">
         <v>183</v>
@@ -2334,13 +2334,13 @@
         <v>100</v>
       </c>
       <c r="C38" s="31" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D38" s="34" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E38" s="31" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F38" s="31"/>
     </row>
@@ -2352,10 +2352,10 @@
         <v>174</v>
       </c>
       <c r="C39" s="31" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D39" s="31" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E39" s="31"/>
       <c r="F39" s="31"/>
@@ -2371,10 +2371,10 @@
         <v>194</v>
       </c>
       <c r="D40" s="34" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E40" s="34" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F40" s="31"/>
     </row>
@@ -2408,7 +2408,7 @@
         <v>12</v>
       </c>
       <c r="E42" s="34" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F42" s="31"/>
     </row>
@@ -2426,7 +2426,7 @@
         <v>64</v>
       </c>
       <c r="E43" s="31" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F43" s="31"/>
     </row>
@@ -2441,7 +2441,7 @@
         <v>144</v>
       </c>
       <c r="D44" s="31" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E44" s="31"/>
       <c r="F44" s="31"/>
@@ -2460,7 +2460,7 @@
         <v>104</v>
       </c>
       <c r="E45" s="31" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F45" s="31"/>
     </row>
@@ -2507,7 +2507,7 @@
         <v>157</v>
       </c>
       <c r="D48" s="31" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E48" s="31"/>
       <c r="F48" s="31"/>
@@ -2523,7 +2523,7 @@
         <v>52</v>
       </c>
       <c r="D49" s="31" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E49" s="31"/>
       <c r="F49" s="31"/>
@@ -2539,7 +2539,7 @@
         <v>141</v>
       </c>
       <c r="D50" s="31" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E50" s="31"/>
       <c r="F50" s="31"/>
@@ -2555,7 +2555,7 @@
         <v>154</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E51" s="31"/>
       <c r="F51" s="31"/>
@@ -2571,7 +2571,7 @@
         <v>155</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E52" s="31"/>
       <c r="F52" s="31"/>
@@ -2584,13 +2584,13 @@
         <v>55</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>56</v>
       </c>
       <c r="E53" s="34" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F53" s="31"/>
     </row>
@@ -2618,7 +2618,7 @@
         <v>124</v>
       </c>
       <c r="C55" s="31" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D55" s="31" t="s">
         <v>186</v>
@@ -2640,7 +2640,7 @@
         <v>105</v>
       </c>
       <c r="E56" s="31" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F56" s="31"/>
     </row>
@@ -2668,10 +2668,10 @@
         <v>122</v>
       </c>
       <c r="C58" s="31" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D58" s="31" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E58" s="31"/>
       <c r="F58" s="31"/>
@@ -2684,7 +2684,7 @@
         <v>125</v>
       </c>
       <c r="C59" s="31" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D59" s="34" t="s">
         <v>128</v>
@@ -2700,7 +2700,7 @@
         <v>126</v>
       </c>
       <c r="C60" s="31" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D60" s="34" t="s">
         <v>129</v>
@@ -2716,14 +2716,14 @@
         <v>28</v>
       </c>
       <c r="C61" s="31" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D61" s="31" t="s">
         <v>41</v>
       </c>
       <c r="E61" s="31"/>
       <c r="F61" s="34" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="56" x14ac:dyDescent="0.2">
@@ -2734,14 +2734,14 @@
         <v>30</v>
       </c>
       <c r="C62" s="31" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D62" s="31" t="s">
         <v>42</v>
       </c>
       <c r="E62" s="31"/>
       <c r="F62" s="34" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
@@ -2752,7 +2752,7 @@
         <v>31</v>
       </c>
       <c r="C63" s="31" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D63" s="31" t="s">
         <v>43</v>
@@ -2768,7 +2768,7 @@
         <v>32</v>
       </c>
       <c r="C64" s="31" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D64" s="31" t="s">
         <v>44</v>
@@ -2784,7 +2784,7 @@
         <v>33</v>
       </c>
       <c r="C65" s="31" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D65" s="31" t="s">
         <v>45</v>
@@ -2800,7 +2800,7 @@
         <v>34</v>
       </c>
       <c r="C66" s="31" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D66" s="31" t="s">
         <v>46</v>
@@ -2822,7 +2822,7 @@
         <v>187</v>
       </c>
       <c r="E67" s="31" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F67" s="31"/>
     </row>
@@ -2834,7 +2834,7 @@
         <v>35</v>
       </c>
       <c r="C68" s="31" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D68" s="31" t="s">
         <v>49</v>
@@ -2850,7 +2850,7 @@
         <v>36</v>
       </c>
       <c r="C69" s="31" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D69" s="31" t="s">
         <v>50</v>
@@ -2866,7 +2866,7 @@
         <v>37</v>
       </c>
       <c r="C70" s="31" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D70" s="31" t="s">
         <v>51</v>
@@ -2882,7 +2882,7 @@
         <v>188</v>
       </c>
       <c r="C71" s="31" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D71" s="31" t="s">
         <v>189</v>
@@ -2898,7 +2898,7 @@
         <v>190</v>
       </c>
       <c r="C72" s="31" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D72" s="31" t="s">
         <v>191</v>
@@ -2914,7 +2914,7 @@
         <v>130</v>
       </c>
       <c r="C73" s="31" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D73" s="31" t="s">
         <v>131</v>
@@ -2978,27 +2978,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="45" t="s">
         <v>175</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
       <c r="D1" s="10" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
       <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="46"/>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
+      <c r="A3" s="45"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
       <c r="D3" s="11" t="s">
         <v>179</v>
       </c>
@@ -3044,27 +3044,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="45" t="s">
         <v>164</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
       <c r="D1" s="10" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
       <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="46"/>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
+      <c r="A3" s="45"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
       <c r="D3" s="11" t="s">
         <v>25</v>
       </c>
@@ -44056,27 +44056,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="45" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
       <c r="D1" s="5" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:53" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
       <c r="D2" s="6"/>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.2">
-      <c r="A3" s="46"/>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
+      <c r="A3" s="45"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
       <c r="D3" s="6" t="s">
         <v>25</v>
       </c>
@@ -44121,7 +44121,7 @@
         <v>117</v>
       </c>
       <c r="H5" s="39" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="I5" s="39" t="s">
         <v>167</v>
@@ -44297,7 +44297,7 @@
       <formula1>"Idividual, Composite, Mean, SD, Equation"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M6:M10000" xr:uid="{D77F31B9-1615-2E41-A61E-3373EC534A30}">
-      <formula1>"fry, larva, nymph, pupa, juvenile, adult "</formula1>
+      <formula1>"egg, fry, larva, nymph, pupa, juvenile, adult "</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L6:L10000" xr:uid="{8E9C54B4-F117-8C42-9731-37E4B818ABAE}">
       <formula1>"male, female, unknown, both"</formula1>

</xml_diff>

<commit_message>
Changed template to use Individual as it was missing the n
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v21.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v21.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8217666-37A6-3142-BA7D-5514BAC9F65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C63A628-57D8-3148-9557-7797C8A71C65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
@@ -44159,7 +44159,7 @@
       <c r="S5" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="T5" s="40" t="s">
+      <c r="T5" s="41" t="s">
         <v>192</v>
       </c>
       <c r="U5" s="40" t="s">
@@ -44293,9 +44293,6 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU6:AU10000" xr:uid="{0DD4FFBC-3D6E-914E-8511-DDD8F03F7232}">
       <formula1>"bulk, lipid free"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T6:T10000" xr:uid="{FE3B4961-9F35-5942-85C0-C97B5B164DB5}">
-      <formula1>"Idividual, Composite, Mean, SD, Equation"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M6:M10000" xr:uid="{D77F31B9-1615-2E41-A61E-3373EC534A30}">
       <formula1>"egg, fry, larva, nymph, pupa, juvenile, adult "</formula1>
     </dataValidation>
@@ -44308,6 +44305,9 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V6:V100000" xr:uid="{1DF4AB3C-A284-C746-89D8-9719DCC064CE}">
       <formula1>"belly flap, blood, carcass, cleithra, eye lens, egg, fin, gonad, heart, liver, muscle, otolith, scales, spine, stomach, viscera, whole body, whole body (gonads removed), whole body (stomach removed)"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T6:T100000" xr:uid="{E1E54910-66C6-C048-9B46-4FB39063E14B}">
+      <formula1>"Individual, Composite, Mean, SD, Equation"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>